<commit_message>
Add Aneesh Kumar (AOT0006) with photo to Bigg Bear employee list
</commit_message>
<xml_diff>
--- a/Bigg Bear- Employee list (1).xlsx
+++ b/Bigg Bear- Employee list (1).xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>S. No.</t>
   </si>
@@ -84,6 +84,12 @@
   </si>
   <si>
     <t>AOT0005</t>
+  </si>
+  <si>
+    <t>Aneesh Kumar</t>
+  </si>
+  <si>
+    <t>AOT0006</t>
   </si>
 </sst>
 </file>
@@ -474,6 +480,50 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3803650" y="3200400"/>
+          <a:ext cx="539750" cy="748125"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>654050</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>24225</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A1B2C3D-4E5F-4071-8293-A4B5C6D7E8F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3803650" y="3962400"/>
           <a:ext cx="539750" cy="748125"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -771,7 +821,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{385038A2-A74E-41F2-9D08-E78D0DC5FA4D}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="11"/>
@@ -933,12 +983,39 @@
       <c r="A21" s="7"/>
       <c r="E21" s="6"/>
     </row>
-    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="8"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="10"/>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="5">
+        <v>6</v>
+      </c>
+      <c r="B22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22">
+        <v>6306177706</v>
+      </c>
+      <c r="E22" s="6"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="7"/>
+      <c r="E23" s="6"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="7"/>
+      <c r="E24" s="6"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="7"/>
+      <c r="E25" s="6"/>
+    </row>
+    <row r="26" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="8"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>